<commit_message>
feat: concluir importador sintético v1
</commit_message>
<xml_diff>
--- a/tests/fixtures/planilha_importacao_v1_sintetica.xlsx
+++ b/tests/fixtures/planilha_importacao_v1_sintetica.xlsx
@@ -744,16 +744,81 @@
           <t>S</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>não</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>10/02/1980</t>
@@ -766,7 +831,37 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>feminino</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>parda</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Rua Sintética, 1</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Cidade Sintética</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>(00) 0000-0000</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>quilombola</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -779,11 +874,151 @@
           <t>hospital</t>
         </is>
       </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>ELISA</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>IFI</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>02/07/2026</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>HAI</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>cardiaca</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>arritmia sintética</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>alteração sintética</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>outra sintética</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="BI2" t="inlineStr">
         <is>
           <t>92,5</t>
         </is>
       </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="BL2" t="inlineStr">
         <is>
           <t>55</t>
@@ -804,6 +1039,91 @@
           <t>30/07/2026</t>
         </is>
       </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="BQ2" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="BY2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="CE2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="CF2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="CG2" t="inlineStr">
         <is>
           <t>sim</t>
@@ -826,7 +1146,12 @@
       </c>
       <c r="CK2" t="inlineStr">
         <is>
-          <t>eco solicitado</t>
+          <t>eco sintético</t>
+        </is>
+      </c>
+      <c r="CL2" t="inlineStr">
+        <is>
+          <t>55%</t>
         </is>
       </c>
       <c r="CN2" t="inlineStr">
@@ -834,6 +1159,41 @@
           <t>hemograma trazido</t>
         </is>
       </c>
+      <c r="CO2" t="inlineStr">
+        <is>
+          <t>imagem sintética</t>
+        </is>
+      </c>
+      <c r="CP2" t="inlineStr">
+        <is>
+          <t>holter sintético</t>
+        </is>
+      </c>
+      <c r="CQ2" t="inlineStr">
+        <is>
+          <t>endoscopia sintética</t>
+        </is>
+      </c>
+      <c r="CR2" t="inlineStr">
+        <is>
+          <t>colonoscopia sintética</t>
+        </is>
+      </c>
+      <c r="CS2" t="inlineStr">
+        <is>
+          <t>teste sintético</t>
+        </is>
+      </c>
+      <c r="CT2" t="inlineStr">
+        <is>
+          <t>mapa sintético</t>
+        </is>
+      </c>
+      <c r="CU2" t="inlineStr">
+        <is>
+          <t>outro exame sintético</t>
+        </is>
+      </c>
       <c r="CW2" t="inlineStr">
         <is>
           <t>hemograma trazido</t>
@@ -841,7 +1201,42 @@
       </c>
       <c r="CX2" t="inlineStr">
         <is>
-          <t>eco solicitado</t>
+          <t>eco sintético</t>
+        </is>
+      </c>
+      <c r="CY2" t="inlineStr">
+        <is>
+          <t>imagem sintética</t>
+        </is>
+      </c>
+      <c r="CZ2" t="inlineStr">
+        <is>
+          <t>holter sintético</t>
+        </is>
+      </c>
+      <c r="DA2" t="inlineStr">
+        <is>
+          <t>endoscopia sintética</t>
+        </is>
+      </c>
+      <c r="DB2" t="inlineStr">
+        <is>
+          <t>colonoscopia sintética</t>
+        </is>
+      </c>
+      <c r="DC2" t="inlineStr">
+        <is>
+          <t>teste sintético</t>
+        </is>
+      </c>
+      <c r="DD2" t="inlineStr">
+        <is>
+          <t>mapa sintético</t>
+        </is>
+      </c>
+      <c r="DE2" t="inlineStr">
+        <is>
+          <t>outro exame sintético</t>
         </is>
       </c>
       <c r="DF2" t="inlineStr">
@@ -882,6 +1277,81 @@
       <c r="DP2" t="inlineStr">
         <is>
           <t>sami_trop_aim3</t>
+        </is>
+      </c>
+      <c r="DR2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="DS2" t="inlineStr">
+        <is>
+          <t>NOT-SINT-1</t>
+        </is>
+      </c>
+      <c r="DT2" t="inlineStr">
+        <is>
+          <t>justificativa sintética</t>
+        </is>
+      </c>
+      <c r="DU2" t="inlineStr">
+        <is>
+          <t>1,70</t>
+        </is>
+      </c>
+      <c r="DV2" t="inlineStr">
+        <is>
+          <t>70,5</t>
+        </is>
+      </c>
+      <c r="DW2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="DX2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DY2" t="inlineStr">
+        <is>
+          <t>98%</t>
+        </is>
+      </c>
+      <c r="DZ2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="EA2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="EB2" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="EC2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="ED2" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
+        </is>
+      </c>
+      <c r="EE2" t="inlineStr">
+        <is>
+          <t>causa sintética</t>
+        </is>
+      </c>
+      <c r="EI2" t="inlineStr">
+        <is>
+          <t>B1</t>
         </is>
       </c>
       <c r="EJ2" t="inlineStr">
@@ -1059,6 +1529,43 @@
       <c r="DF8" t="inlineStr">
         <is>
           <t>talvez</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>P-ATOM</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Falha Atômica</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>07/07/1987</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Endereço que deve sofrer rollback</t>
+        </is>
+      </c>
+      <c r="DR9" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="DT9" t="inlineStr">
+        <is>
+          <t>contradição sintética</t>
         </is>
       </c>
     </row>
@@ -1777,29 +2284,79 @@
           <t>08/08/1988</t>
         </is>
       </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="AE2" t="inlineStr">
         <is>
           <t>não</t>
         </is>
       </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>01/01/2020</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="CC2" t="inlineStr">
         <is>
           <t>não</t>
         </is>
       </c>
+      <c r="CI2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="CJ2" t="inlineStr">
         <is>
           <t>solicitar painel</t>
         </is>
       </c>
+      <c r="CR2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="CS2" t="inlineStr">
         <is>
           <t>solicitar painel</t>
         </is>
       </c>
+      <c r="DI2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="DK2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="DM2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="EB2" t="inlineStr">
         <is>
           <t>texto parcial preservado</t>
+        </is>
+      </c>
+      <c r="EC2" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="ED2" t="inlineStr">
+        <is>
+          <t>texto sintético</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: reconciliar tratamento BZN consolidado no importador
</commit_message>
<xml_diff>
--- a/tests/fixtures/planilha_importacao_v1_sintetica.xlsx
+++ b/tests/fixtures/planilha_importacao_v1_sintetica.xlsx
@@ -1406,6 +1406,41 @@
           <t>resultado eco segundo atendimento</t>
         </is>
       </c>
+      <c r="DF3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="DG3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="DH3" t="inlineStr">
+        <is>
+          <t>56 dias</t>
+        </is>
+      </c>
+      <c r="DI3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="DJ3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="DK3" t="inlineStr">
+        <is>
+          <t>01/06/2025</t>
+        </is>
+      </c>
+      <c r="DN3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1433,6 +1468,16 @@
           <t>03/03/1990</t>
         </is>
       </c>
+      <c r="DJ4" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="DN4" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1566,6 +1611,122 @@
       <c r="DT9" t="inlineStr">
         <is>
           <t>contradição sintética</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>P-NOVO</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Carlos Sintético</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>03/03/1990</t>
+        </is>
+      </c>
+      <c r="DF10" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="DH10" t="inlineStr">
+        <is>
+          <t>7 dias</t>
+        </is>
+      </c>
+      <c r="DI10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>P-NOVO</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Carlos Sintético</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>03/03/1990</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Endereço sintético da linha BZN rejeitada</t>
+        </is>
+      </c>
+      <c r="DF11" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="DG11" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="DH11" t="inlineStr">
+        <is>
+          <t>1 semana</t>
+        </is>
+      </c>
+      <c r="DI11" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>P-NOVO</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Carlos Sintético</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>03/03/1990</t>
+        </is>
+      </c>
+      <c r="DF12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="DH12" t="inlineStr">
+        <is>
+          <t>1 semana</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: evoluir importador e otimizar workflow de validação
</commit_message>
<xml_diff>
--- a/tests/fixtures/planilha_importacao_v1_sintetica.xlsx
+++ b/tests/fixtures/planilha_importacao_v1_sintetica.xlsx
@@ -749,11 +749,6 @@
           <t>não</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>não</t>
@@ -1439,6 +1434,11 @@
       <c r="DN3" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="EF3" t="inlineStr">
+        <is>
+          <t>pendência sintética conflitante</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: cobrir promoções e reprocessamento do importador
</commit_message>
<xml_diff>
--- a/tests/fixtures/planilha_importacao_v1_sintetica.xlsx
+++ b/tests/fixtures/planilha_importacao_v1_sintetica.xlsx
@@ -1264,9 +1264,19 @@
           <t>01/06/2025</t>
         </is>
       </c>
+      <c r="DM2" t="inlineStr">
+        <is>
+          <t>15/07/2025</t>
+        </is>
+      </c>
       <c r="DN2" t="inlineStr">
         <is>
           <t>não</t>
+        </is>
+      </c>
+      <c r="DO2" t="inlineStr">
+        <is>
+          <t>30/08/2025</t>
         </is>
       </c>
       <c r="DP2" t="inlineStr">

</xml_diff>